<commit_message>
Versão enxuta da planilha (Painel, Premissas, Meu Mês, Projeção)
- Mesa_Agil_Enxuta.xlsx: ~15 campos para preencher uma vez e 6 números
  por mês na aba Meu Mês, que compara o real com o planejado.
- estilo_app.py: estilo do design system do app compartilhado pelas
  duas planilhas (a completa continua idêntica).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011pEscwW9GNGpmNb8Mg2awf
</commit_message>
<xml_diff>
--- a/Mesa_Agil_Financeiro.xlsx
+++ b/Mesa_Agil_Financeiro.xlsx
@@ -1392,47 +1392,47 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="172" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2305,11 +2305,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="74872893"/>
-        <c:axId val="14224493"/>
+        <c:axId val="31108518"/>
+        <c:axId val="68067138"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74872893"/>
+        <c:axId val="31108518"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2341,7 +2341,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14224493"/>
+        <c:crossAx val="68067138"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2349,7 +2349,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14224493"/>
+        <c:axId val="68067138"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2391,7 +2391,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74872893"/>
+        <c:crossAx val="31108518"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2700,11 +2700,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="4794764"/>
-        <c:axId val="6325737"/>
+        <c:axId val="57768776"/>
+        <c:axId val="25473196"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="4794764"/>
+        <c:axId val="57768776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2736,7 +2736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6325737"/>
+        <c:crossAx val="25473196"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2744,7 +2744,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6325737"/>
+        <c:axId val="25473196"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2786,7 +2786,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4794764"/>
+        <c:crossAx val="57768776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3071,11 +3071,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="498040"/>
-        <c:axId val="95670399"/>
+        <c:axId val="65918378"/>
+        <c:axId val="84995692"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="498040"/>
+        <c:axId val="65918378"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3107,7 +3107,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95670399"/>
+        <c:crossAx val="84995692"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3115,7 +3115,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95670399"/>
+        <c:axId val="84995692"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3157,7 +3157,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="498040"/>
+        <c:crossAx val="65918378"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3670,11 +3670,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="75670372"/>
-        <c:axId val="52594944"/>
+        <c:axId val="97090097"/>
+        <c:axId val="80415619"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="75670372"/>
+        <c:axId val="97090097"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3706,7 +3706,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52594944"/>
+        <c:crossAx val="80415619"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3714,7 +3714,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52594944"/>
+        <c:axId val="80415619"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3756,7 +3756,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75670372"/>
+        <c:crossAx val="97090097"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4509,11 +4509,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="52385952"/>
-        <c:axId val="15446512"/>
+        <c:axId val="25061169"/>
+        <c:axId val="34720646"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52385952"/>
+        <c:axId val="25061169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4545,7 +4545,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15446512"/>
+        <c:crossAx val="34720646"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4553,7 +4553,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15446512"/>
+        <c:axId val="34720646"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4595,7 +4595,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52385952"/>
+        <c:crossAx val="25061169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5348,11 +5348,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="20547732"/>
-        <c:axId val="5007814"/>
+        <c:axId val="13942583"/>
+        <c:axId val="71011309"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="20547732"/>
+        <c:axId val="13942583"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5384,7 +5384,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5007814"/>
+        <c:crossAx val="71011309"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5392,7 +5392,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5007814"/>
+        <c:axId val="71011309"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5434,7 +5434,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20547732"/>
+        <c:crossAx val="13942583"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6187,11 +6187,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="46232707"/>
-        <c:axId val="54995688"/>
+        <c:axId val="89483661"/>
+        <c:axId val="44752945"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="46232707"/>
+        <c:axId val="89483661"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6223,7 +6223,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54995688"/>
+        <c:crossAx val="44752945"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6231,7 +6231,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54995688"/>
+        <c:axId val="44752945"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6273,7 +6273,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46232707"/>
+        <c:crossAx val="89483661"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>